<commit_message>
change theme sky blue to brand and add field template excel
</commit_message>
<xml_diff>
--- a/public/Add_Users_Template.xlsx
+++ b/public/Add_Users_Template.xlsx
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:AA1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="12.796875" customWidth="1" min="1" max="4"/>
@@ -466,62 +466,137 @@
     <row r="1" ht="15.6" customHeight="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>คำนำหน้า</t>
+          <t xml:space="preserve">คำนำหน้า</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>ชื่อ</t>
+          <t xml:space="preserve">ชื่อ</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>นามสกุล</t>
+          <t xml:space="preserve">นามสกุล</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>อีเมล</t>
+          <t xml:space="preserve">อีเมล</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>เบอร์ติดต่อ</t>
+          <t xml:space="preserve">เบอร์ติดต่อ</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>ตำแหน่งงาน</t>
+          <t xml:space="preserve">ตำแหน่งงาน</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>เลขที่ตำแหน่ง</t>
+          <t xml:space="preserve">เลขที่ตำแหน่ง</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>วันที่บรรจุ</t>
+          <t xml:space="preserve">วันที่บรรจุ</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>สายงาน</t>
+          <t xml:space="preserve">สายงาน</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>สาขา</t>
+          <t xml:space="preserve">สาขา</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>ประเภทบุคคล</t>
+          <t xml:space="preserve">ประเภทบุคคล</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>บทบาท</t>
+          <t xml:space="preserve">บทบาท</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ลาป่วย (วันคงเหลือ)</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ลาคลอดบุตร (วันคงเหลือ)</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ลากิจส่วนตัว (วันคงเหลือ)</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ลาพักผ่อน (วันคงเหลือ)</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ลาอุปสมบท (วันที่ใช้ไปแล้ว)</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ลาตรวจเลือก/เตรียมพล (วันที่ใช้ไปแล้ว)</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ลาไปศึกษา (วันคงเหลือ)</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ลาช่วยเหลือภริยาที่คลอดบุตร (วันคงเหลือ)</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ลาฟื้นฟูสมรรถภาพด้านอาชีพ (วันคงเหลือ)</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ลาถือศีล/ปฏิบัติธรรม สตรี (วันที่ใช้ไปแล้ว)</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ลาองค์การระหว่างประเทศ (วันที่ใช้ไปแล้ว)</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ลาติดตามคู่สมรส (วันคงเหลือ)</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ลาประกอบพิธีฮัจย์ (วันที่ใช้ไปแล้ว)</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ลาฝึกอบรม/วิจัย/ดูงาน (วันคงเหลือ)</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ไปราชการ (วันที่ใช้ไปแล้ว)</t>
         </is>
       </c>
     </row>

</xml_diff>